<commit_message>
Publish intermission Period TOI workbook
</commit_message>
<xml_diff>
--- a/clarkson_intermission_toi_48d1d66f-0466-44ae-8987-278e8c64a996_p2.xlsx
+++ b/clarkson_intermission_toi_48d1d66f-0466-44ae-8987-278e8c64a996_p2.xlsx
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>449.4616979999998</v>
+        <v>449.4616759999999</v>
       </c>
       <c r="H3" t="n">
         <v>816275</v>
@@ -568,7 +568,7 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>399.9501730000001</v>
+        <v>399.950193</v>
       </c>
       <c r="H4" t="n">
         <v>816596</v>
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>397.6676129999998</v>
+        <v>397.667603</v>
       </c>
       <c r="H5" t="n">
         <v>816647</v>
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>388.9927709999998</v>
+        <v>388.992801</v>
       </c>
       <c r="H7" t="n">
         <v>821897</v>
@@ -880,7 +880,7 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>325.6053589999999</v>
+        <v>325.605349</v>
       </c>
       <c r="H12" t="n">
         <v>824230</v>
@@ -1549,16 +1549,16 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>31</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Sydney Lamb</t>
+          <t>Senkova Aneta</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>821897</v>
+        <v>801351</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1566,17 +1566,17 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>1233.0256</v>
+        <v>1200.5223</v>
       </c>
       <c r="H7" t="n">
-        <v>1306.8716</v>
+        <v>2400</v>
       </c>
       <c r="I7" t="n">
-        <v>73.846</v>
+        <v>1199.478</v>
       </c>
       <c r="J7" s="1" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>19.59</t>
         </is>
       </c>
       <c r="K7" t="b">
@@ -1594,16 +1594,16 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Ciara Lang</t>
+          <t>Sydney Lamb</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>906527</v>
+        <v>821897</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1639,16 +1639,16 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>19</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Jessie Pellerin</t>
+          <t>Ciara Lang</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>801538</v>
+        <v>906527</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1659,14 +1659,14 @@
         <v>1233.0256</v>
       </c>
       <c r="H9" t="n">
-        <v>1259.7705</v>
+        <v>1306.8716</v>
       </c>
       <c r="I9" t="n">
-        <v>26.745</v>
+        <v>73.846</v>
       </c>
       <c r="J9" s="1" t="inlineStr">
         <is>
-          <t>0.27</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="K9" t="b">
@@ -1684,16 +1684,16 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>27</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Isa Goettl</t>
+          <t>Jessie Pellerin</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>816244</v>
+        <v>801538</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1729,16 +1729,16 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Janelle Evans</t>
+          <t>Isa Goettl</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>818654</v>
+        <v>816244</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -1774,16 +1774,16 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Raedyn Spademan</t>
+          <t>Janelle Evans</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>816647</v>
+        <v>818654</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -1791,17 +1791,17 @@
         </is>
       </c>
       <c r="G12" t="n">
+        <v>1233.0256</v>
+      </c>
+      <c r="H12" t="n">
         <v>1259.7705</v>
       </c>
-      <c r="H12" t="n">
-        <v>1306.8066</v>
-      </c>
       <c r="I12" t="n">
-        <v>47.036</v>
+        <v>26.745</v>
       </c>
       <c r="J12" s="1" t="inlineStr">
         <is>
-          <t>0.47</t>
+          <t>0.27</t>
         </is>
       </c>
       <c r="K12" t="b">
@@ -1819,16 +1819,16 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>18</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Shelby Laidlaw</t>
+          <t>Raedyn Spademan</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>816596</v>
+        <v>816647</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -1864,16 +1864,16 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>28</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Layla Matthew</t>
+          <t>Shelby Laidlaw</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>847129</v>
+        <v>816596</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1909,16 +1909,16 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Gabrielle Lalonde</t>
+          <t>Layla Matthew</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>856725</v>
+        <v>847129</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1926,17 +1926,17 @@
         </is>
       </c>
       <c r="G15" t="n">
+        <v>1259.7705</v>
+      </c>
+      <c r="H15" t="n">
         <v>1306.8066</v>
       </c>
-      <c r="H15" t="n">
-        <v>1385.4287</v>
-      </c>
       <c r="I15" t="n">
-        <v>78.622</v>
+        <v>47.036</v>
       </c>
       <c r="J15" s="1" t="inlineStr">
         <is>
-          <t>1.19</t>
+          <t>0.47</t>
         </is>
       </c>
       <c r="K15" t="b">
@@ -1954,16 +1954,16 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Abby Richardson</t>
+          <t>Gabrielle Lalonde</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>824230</v>
+        <v>856725</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1999,16 +1999,16 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Paige Wallace</t>
+          <t>Abby Richardson</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>822075</v>
+        <v>824230</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -2019,14 +2019,14 @@
         <v>1306.8066</v>
       </c>
       <c r="H17" t="n">
-        <v>1349.9097</v>
+        <v>1385.4287</v>
       </c>
       <c r="I17" t="n">
-        <v>43.103</v>
+        <v>78.622</v>
       </c>
       <c r="J17" s="1" t="inlineStr">
         <is>
-          <t>0.43</t>
+          <t>1.19</t>
         </is>
       </c>
       <c r="K17" t="b">
@@ -2044,16 +2044,16 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Kaitlyn Mallette</t>
+          <t>Paige Wallace</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>847128</v>
+        <v>822075</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -2061,17 +2061,17 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>1306.8716</v>
+        <v>1306.8066</v>
       </c>
       <c r="H18" t="n">
-        <v>1352.4473</v>
+        <v>1349.9097</v>
       </c>
       <c r="I18" t="n">
-        <v>45.576</v>
+        <v>43.103</v>
       </c>
       <c r="J18" s="1" t="inlineStr">
         <is>
-          <t>0.46</t>
+          <t>0.43</t>
         </is>
       </c>
       <c r="K18" t="b">
@@ -2089,16 +2089,16 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>11</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Morgan Walton</t>
+          <t>Kaitlyn Mallette</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>822077</v>
+        <v>847128</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -2109,14 +2109,14 @@
         <v>1306.8716</v>
       </c>
       <c r="H19" t="n">
-        <v>1385.4287</v>
+        <v>1352.4473</v>
       </c>
       <c r="I19" t="n">
-        <v>78.557</v>
+        <v>45.576</v>
       </c>
       <c r="J19" s="1" t="inlineStr">
         <is>
-          <t>1.19</t>
+          <t>0.46</t>
         </is>
       </c>
       <c r="K19" t="b">
@@ -2134,16 +2134,16 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Sara Manness</t>
+          <t>Morgan Walton</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>801530</v>
+        <v>822077</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -2151,17 +2151,17 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>1349.9097</v>
+        <v>1306.8716</v>
       </c>
       <c r="H20" t="n">
         <v>1385.4287</v>
       </c>
       <c r="I20" t="n">
-        <v>35.519</v>
+        <v>78.557</v>
       </c>
       <c r="J20" s="1" t="inlineStr">
         <is>
-          <t>0.36</t>
+          <t>1.19</t>
         </is>
       </c>
       <c r="K20" t="b">
@@ -2179,16 +2179,16 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>26</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Keira Hurry</t>
+          <t>Sara Manness</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>816275</v>
+        <v>801530</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -2196,17 +2196,17 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>1352.4473</v>
+        <v>1349.9097</v>
       </c>
       <c r="H21" t="n">
-        <v>1414.8298</v>
+        <v>1385.4287</v>
       </c>
       <c r="I21" t="n">
-        <v>62.383</v>
+        <v>35.519</v>
       </c>
       <c r="J21" s="1" t="inlineStr">
         <is>
-          <t>1.02</t>
+          <t>0.36</t>
         </is>
       </c>
       <c r="K21" t="b">
@@ -2224,16 +2224,16 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Kate Manness</t>
+          <t>Keira Hurry</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>835282</v>
+        <v>816275</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -2241,17 +2241,17 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>1385.4287</v>
+        <v>1352.4473</v>
       </c>
       <c r="H22" t="n">
-        <v>1422.9797</v>
+        <v>1414.8298</v>
       </c>
       <c r="I22" t="n">
-        <v>37.551</v>
+        <v>62.383</v>
       </c>
       <c r="J22" s="1" t="inlineStr">
         <is>
-          <t>0.38</t>
+          <t>1.02</t>
         </is>
       </c>
       <c r="K22" t="b">
@@ -2269,16 +2269,16 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>24</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Janelle Evans</t>
+          <t>Kate Manness</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>818654</v>
+        <v>835282</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -2289,14 +2289,14 @@
         <v>1385.4287</v>
       </c>
       <c r="H23" t="n">
-        <v>1442.7845</v>
+        <v>1422.9797</v>
       </c>
       <c r="I23" t="n">
-        <v>57.356</v>
+        <v>37.551</v>
       </c>
       <c r="J23" s="1" t="inlineStr">
         <is>
-          <t>0.57</t>
+          <t>0.38</t>
         </is>
       </c>
       <c r="K23" t="b">
@@ -2314,16 +2314,16 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>17</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Jessie Pellerin</t>
+          <t>Janelle Evans</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>801538</v>
+        <v>818654</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -2334,14 +2334,14 @@
         <v>1385.4287</v>
       </c>
       <c r="H24" t="n">
-        <v>1430.5482</v>
+        <v>1442.7845</v>
       </c>
       <c r="I24" t="n">
-        <v>45.12</v>
+        <v>57.356</v>
       </c>
       <c r="J24" s="1" t="inlineStr">
         <is>
-          <t>0.45</t>
+          <t>0.57</t>
         </is>
       </c>
       <c r="K24" t="b">
@@ -2359,16 +2359,16 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>27</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Isa Goettl</t>
+          <t>Jessie Pellerin</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>816244</v>
+        <v>801538</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -2379,14 +2379,14 @@
         <v>1385.4287</v>
       </c>
       <c r="H25" t="n">
-        <v>1442.7845</v>
+        <v>1430.5482</v>
       </c>
       <c r="I25" t="n">
-        <v>57.356</v>
+        <v>45.12</v>
       </c>
       <c r="J25" s="1" t="inlineStr">
         <is>
-          <t>0.57</t>
+          <t>0.45</t>
         </is>
       </c>
       <c r="K25" t="b">
@@ -2404,16 +2404,16 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Ciara Lang</t>
+          <t>Isa Goettl</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>906527</v>
+        <v>816244</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -2421,17 +2421,17 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>1414.8298</v>
+        <v>1385.4287</v>
       </c>
       <c r="H26" t="n">
-        <v>1443.9337</v>
+        <v>1442.7845</v>
       </c>
       <c r="I26" t="n">
-        <v>29.104</v>
+        <v>57.356</v>
       </c>
       <c r="J26" s="1" t="inlineStr">
         <is>
-          <t>0.29</t>
+          <t>0.57</t>
         </is>
       </c>
       <c r="K26" t="b">
@@ -2449,16 +2449,16 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>19</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Kaitlyn Mallette</t>
+          <t>Ciara Lang</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>847128</v>
+        <v>906527</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -2466,17 +2466,17 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>1422.9797</v>
+        <v>1414.8298</v>
       </c>
       <c r="H27" t="n">
-        <v>1486.886</v>
+        <v>1443.9337</v>
       </c>
       <c r="I27" t="n">
-        <v>63.906</v>
+        <v>29.104</v>
       </c>
       <c r="J27" s="1" t="inlineStr">
         <is>
-          <t>1.04</t>
+          <t>0.29</t>
         </is>
       </c>
       <c r="K27" t="b">
@@ -2494,16 +2494,16 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>11</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Sara Manness</t>
+          <t>Kaitlyn Mallette</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>801530</v>
+        <v>847128</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -2511,17 +2511,17 @@
         </is>
       </c>
       <c r="G28" t="n">
-        <v>1430.5482</v>
+        <v>1422.9797</v>
       </c>
       <c r="H28" t="n">
         <v>1486.886</v>
       </c>
       <c r="I28" t="n">
-        <v>56.338</v>
+        <v>63.906</v>
       </c>
       <c r="J28" s="1" t="inlineStr">
         <is>
-          <t>0.56</t>
+          <t>1.04</t>
         </is>
       </c>
       <c r="K28" t="b">
@@ -2539,16 +2539,16 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>26</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Kennedy Sisson</t>
+          <t>Sara Manness</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>891409</v>
+        <v>801530</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -2556,17 +2556,17 @@
         </is>
       </c>
       <c r="G29" t="n">
-        <v>1442.7845</v>
+        <v>1430.5482</v>
       </c>
       <c r="H29" t="n">
         <v>1486.886</v>
       </c>
       <c r="I29" t="n">
-        <v>44.101</v>
+        <v>56.338</v>
       </c>
       <c r="J29" s="1" t="inlineStr">
         <is>
-          <t>0.44</t>
+          <t>0.56</t>
         </is>
       </c>
       <c r="K29" t="b">
@@ -2584,16 +2584,16 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Manon le Scodan</t>
+          <t>Kennedy Sisson</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>811470</v>
+        <v>891409</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -2629,16 +2629,16 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>21</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Sydney Lamb</t>
+          <t>Manon le Scodan</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>821897</v>
+        <v>811470</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -2646,17 +2646,17 @@
         </is>
       </c>
       <c r="G31" t="n">
-        <v>1443.9337</v>
+        <v>1442.7845</v>
       </c>
       <c r="H31" t="n">
         <v>1486.886</v>
       </c>
       <c r="I31" t="n">
-        <v>42.952</v>
+        <v>44.101</v>
       </c>
       <c r="J31" s="1" t="inlineStr">
         <is>
-          <t>0.43</t>
+          <t>0.44</t>
         </is>
       </c>
       <c r="K31" t="b">
@@ -2674,16 +2674,16 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Keira Hurry</t>
+          <t>Sydney Lamb</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>816275</v>
+        <v>821897</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -2691,17 +2691,17 @@
         </is>
       </c>
       <c r="G32" t="n">
+        <v>1443.9337</v>
+      </c>
+      <c r="H32" t="n">
         <v>1486.886</v>
       </c>
-      <c r="H32" t="n">
-        <v>1546.2128</v>
-      </c>
       <c r="I32" t="n">
-        <v>59.327</v>
+        <v>42.952</v>
       </c>
       <c r="J32" s="1" t="inlineStr">
         <is>
-          <t>0.59</t>
+          <t>0.43</t>
         </is>
       </c>
       <c r="K32" t="b">
@@ -2719,16 +2719,16 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Kate Manness</t>
+          <t>Keira Hurry</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>835282</v>
+        <v>816275</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -2764,16 +2764,16 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>24</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Layla Matthew</t>
+          <t>Kate Manness</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>847129</v>
+        <v>835282</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -2784,14 +2784,14 @@
         <v>1486.886</v>
       </c>
       <c r="H34" t="n">
-        <v>1543.1936</v>
+        <v>1546.2128</v>
       </c>
       <c r="I34" t="n">
-        <v>56.308</v>
+        <v>59.327</v>
       </c>
       <c r="J34" s="1" t="inlineStr">
         <is>
-          <t>0.56</t>
+          <t>0.59</t>
         </is>
       </c>
       <c r="K34" t="b">
@@ -2809,16 +2809,16 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>15</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Shelby Laidlaw</t>
+          <t>Layla Matthew</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>816596</v>
+        <v>847129</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -2829,14 +2829,14 @@
         <v>1486.886</v>
       </c>
       <c r="H35" t="n">
-        <v>1540.9703</v>
+        <v>1543.1936</v>
       </c>
       <c r="I35" t="n">
-        <v>54.084</v>
+        <v>56.308</v>
       </c>
       <c r="J35" s="1" t="inlineStr">
         <is>
-          <t>0.54</t>
+          <t>0.56</t>
         </is>
       </c>
       <c r="K35" t="b">
@@ -2854,16 +2854,16 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>28</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Raedyn Spademan</t>
+          <t>Shelby Laidlaw</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>816647</v>
+        <v>816596</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -2874,14 +2874,14 @@
         <v>1486.886</v>
       </c>
       <c r="H36" t="n">
-        <v>1548.9387</v>
+        <v>1540.9703</v>
       </c>
       <c r="I36" t="n">
-        <v>62.053</v>
+        <v>54.084</v>
       </c>
       <c r="J36" s="1" t="inlineStr">
         <is>
-          <t>1.02</t>
+          <t>0.54</t>
         </is>
       </c>
       <c r="K36" t="b">
@@ -2899,16 +2899,16 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>18</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Jessie Pellerin</t>
+          <t>Raedyn Spademan</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>801538</v>
+        <v>816647</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -2916,17 +2916,17 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>1540.9703</v>
+        <v>1486.886</v>
       </c>
       <c r="H37" t="n">
-        <v>1583.9983</v>
+        <v>1548.9387</v>
       </c>
       <c r="I37" t="n">
-        <v>43.028</v>
+        <v>62.053</v>
       </c>
       <c r="J37" s="1" t="inlineStr">
         <is>
-          <t>0.43</t>
+          <t>1.02</t>
         </is>
       </c>
       <c r="K37" t="b">
@@ -2944,16 +2944,16 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>27</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Isa Goettl</t>
+          <t>Jessie Pellerin</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>816244</v>
+        <v>801538</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -2961,17 +2961,17 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>1543.1936</v>
+        <v>1540.9703</v>
       </c>
       <c r="H38" t="n">
         <v>1583.9983</v>
       </c>
       <c r="I38" t="n">
-        <v>40.805</v>
+        <v>43.028</v>
       </c>
       <c r="J38" s="1" t="inlineStr">
         <is>
-          <t>0.41</t>
+          <t>0.43</t>
         </is>
       </c>
       <c r="K38" t="b">
@@ -2989,16 +2989,16 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Morgan Walton</t>
+          <t>Isa Goettl</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>822077</v>
+        <v>816244</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -3006,17 +3006,17 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>1546.2128</v>
+        <v>1543.1936</v>
       </c>
       <c r="H39" t="n">
         <v>1583.9983</v>
       </c>
       <c r="I39" t="n">
-        <v>37.786</v>
+        <v>40.805</v>
       </c>
       <c r="J39" s="1" t="inlineStr">
         <is>
-          <t>0.38</t>
+          <t>0.41</t>
         </is>
       </c>
       <c r="K39" t="b">
@@ -3034,16 +3034,16 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Jaela Carter</t>
+          <t>Morgan Walton</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>856721</v>
+        <v>822077</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -3079,16 +3079,16 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Janelle Evans</t>
+          <t>Jaela Carter</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>818654</v>
+        <v>856721</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -3096,17 +3096,17 @@
         </is>
       </c>
       <c r="G41" t="n">
-        <v>1548.9387</v>
+        <v>1546.2128</v>
       </c>
       <c r="H41" t="n">
         <v>1583.9983</v>
       </c>
       <c r="I41" t="n">
-        <v>35.06</v>
+        <v>37.786</v>
       </c>
       <c r="J41" s="1" t="inlineStr">
         <is>
-          <t>0.35</t>
+          <t>0.38</t>
         </is>
       </c>
       <c r="K41" t="b">
@@ -3124,16 +3124,16 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>17</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Ciara Lang</t>
+          <t>Janelle Evans</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>906527</v>
+        <v>818654</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -3141,17 +3141,17 @@
         </is>
       </c>
       <c r="G42" t="n">
+        <v>1548.9387</v>
+      </c>
+      <c r="H42" t="n">
         <v>1583.9983</v>
       </c>
-      <c r="H42" t="n">
-        <v>1611.8126</v>
-      </c>
       <c r="I42" t="n">
-        <v>27.814</v>
+        <v>35.06</v>
       </c>
       <c r="J42" s="1" t="inlineStr">
         <is>
-          <t>0.28</t>
+          <t>0.35</t>
         </is>
       </c>
       <c r="K42" t="b">
@@ -3169,16 +3169,16 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>19</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Sydney Lamb</t>
+          <t>Ciara Lang</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>821897</v>
+        <v>906527</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -3214,16 +3214,16 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Manon le Scodan</t>
+          <t>Sydney Lamb</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>811470</v>
+        <v>821897</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -3259,16 +3259,16 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>21</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Sara Manness</t>
+          <t>Manon le Scodan</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>801530</v>
+        <v>811470</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -3304,16 +3304,16 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>26</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Kennedy Sisson</t>
+          <t>Sara Manness</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>891409</v>
+        <v>801530</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -3349,16 +3349,16 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>22</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Keira Hurry</t>
+          <t>Kennedy Sisson</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>816275</v>
+        <v>891409</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -3366,17 +3366,17 @@
         </is>
       </c>
       <c r="G47" t="n">
+        <v>1583.9983</v>
+      </c>
+      <c r="H47" t="n">
         <v>1611.8126</v>
       </c>
-      <c r="H47" t="n">
-        <v>1662.9476</v>
-      </c>
       <c r="I47" t="n">
-        <v>51.135</v>
+        <v>27.814</v>
       </c>
       <c r="J47" s="1" t="inlineStr">
         <is>
-          <t>0.51</t>
+          <t>0.28</t>
         </is>
       </c>
       <c r="K47" t="b">
@@ -3394,16 +3394,16 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Kate Manness</t>
+          <t>Keira Hurry</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>835282</v>
+        <v>816275</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -3414,14 +3414,14 @@
         <v>1611.8126</v>
       </c>
       <c r="H48" t="n">
-        <v>1687.3694</v>
+        <v>1662.9476</v>
       </c>
       <c r="I48" t="n">
-        <v>75.557</v>
+        <v>51.135</v>
       </c>
       <c r="J48" s="1" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>0.51</t>
         </is>
       </c>
       <c r="K48" t="b">
@@ -3439,16 +3439,16 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>24</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Janelle Evans</t>
+          <t>Kate Manness</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>818654</v>
+        <v>835282</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -3459,14 +3459,14 @@
         <v>1611.8126</v>
       </c>
       <c r="H49" t="n">
-        <v>1655.3345</v>
+        <v>1687.3694</v>
       </c>
       <c r="I49" t="n">
-        <v>43.522</v>
+        <v>75.557</v>
       </c>
       <c r="J49" s="1" t="inlineStr">
         <is>
-          <t>0.44</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="K49" t="b">
@@ -3484,16 +3484,16 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>17</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Jessie Pellerin</t>
+          <t>Janelle Evans</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>801538</v>
+        <v>818654</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -3504,14 +3504,14 @@
         <v>1611.8126</v>
       </c>
       <c r="H50" t="n">
-        <v>1686.7356</v>
+        <v>1655.3345</v>
       </c>
       <c r="I50" t="n">
-        <v>74.923</v>
+        <v>43.522</v>
       </c>
       <c r="J50" s="1" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>0.44</t>
         </is>
       </c>
       <c r="K50" t="b">
@@ -3529,16 +3529,16 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>27</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Isa Goettl</t>
+          <t>Jessie Pellerin</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>816244</v>
+        <v>801538</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -3549,14 +3549,14 @@
         <v>1611.8126</v>
       </c>
       <c r="H51" t="n">
-        <v>1687.4829</v>
+        <v>1686.7356</v>
       </c>
       <c r="I51" t="n">
-        <v>75.67</v>
+        <v>74.923</v>
       </c>
       <c r="J51" s="1" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="K51" t="b">
@@ -3574,16 +3574,16 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Abby Richardson</t>
+          <t>Isa Goettl</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>824230</v>
+        <v>816244</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -3591,17 +3591,17 @@
         </is>
       </c>
       <c r="G52" t="n">
-        <v>1655.3345</v>
+        <v>1611.8126</v>
       </c>
       <c r="H52" t="n">
-        <v>1743.8737</v>
+        <v>1687.4829</v>
       </c>
       <c r="I52" t="n">
-        <v>88.539</v>
+        <v>75.67</v>
       </c>
       <c r="J52" s="1" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="K52" t="b">
@@ -3619,16 +3619,16 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Morgan Walton</t>
+          <t>Abby Richardson</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>822077</v>
+        <v>824230</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -3636,17 +3636,17 @@
         </is>
       </c>
       <c r="G53" t="n">
-        <v>1662.9476</v>
+        <v>1655.3345</v>
       </c>
       <c r="H53" t="n">
-        <v>1723.5183</v>
+        <v>1743.8737</v>
       </c>
       <c r="I53" t="n">
-        <v>60.571</v>
+        <v>88.539</v>
       </c>
       <c r="J53" s="1" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="K53" t="b">
@@ -3664,16 +3664,16 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Paige Wallace</t>
+          <t>Morgan Walton</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>822075</v>
+        <v>822077</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -3681,17 +3681,17 @@
         </is>
       </c>
       <c r="G54" t="n">
-        <v>1686.7356</v>
+        <v>1662.9476</v>
       </c>
       <c r="H54" t="n">
-        <v>1743.8737</v>
+        <v>1723.5183</v>
       </c>
       <c r="I54" t="n">
-        <v>57.138</v>
+        <v>60.571</v>
       </c>
       <c r="J54" s="1" t="inlineStr">
         <is>
-          <t>0.57</t>
+          <t>1.01</t>
         </is>
       </c>
       <c r="K54" t="b">
@@ -3709,16 +3709,16 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Kaitlyn Mallette</t>
+          <t>Paige Wallace</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>847128</v>
+        <v>822075</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -3726,17 +3726,17 @@
         </is>
       </c>
       <c r="G55" t="n">
-        <v>1687.3694</v>
+        <v>1686.7356</v>
       </c>
       <c r="H55" t="n">
-        <v>1723.5183</v>
+        <v>1743.8737</v>
       </c>
       <c r="I55" t="n">
-        <v>36.149</v>
+        <v>57.138</v>
       </c>
       <c r="J55" s="1" t="inlineStr">
         <is>
-          <t>0.36</t>
+          <t>0.57</t>
         </is>
       </c>
       <c r="K55" t="b">
@@ -3754,16 +3754,16 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>11</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Gabrielle Lalonde</t>
+          <t>Kaitlyn Mallette</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>856725</v>
+        <v>847128</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -3771,17 +3771,17 @@
         </is>
       </c>
       <c r="G56" t="n">
-        <v>1687.4829</v>
+        <v>1687.3694</v>
       </c>
       <c r="H56" t="n">
-        <v>1743.8737</v>
+        <v>1723.5183</v>
       </c>
       <c r="I56" t="n">
-        <v>56.391</v>
+        <v>36.149</v>
       </c>
       <c r="J56" s="1" t="inlineStr">
         <is>
-          <t>0.56</t>
+          <t>0.36</t>
         </is>
       </c>
       <c r="K56" t="b">
@@ -3799,16 +3799,16 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Ciara Lang</t>
+          <t>Gabrielle Lalonde</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>906527</v>
+        <v>856725</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -3816,17 +3816,17 @@
         </is>
       </c>
       <c r="G57" t="n">
-        <v>1723.5183</v>
+        <v>1687.4829</v>
       </c>
       <c r="H57" t="n">
-        <v>1795.7245</v>
+        <v>1743.8737</v>
       </c>
       <c r="I57" t="n">
-        <v>72.206</v>
+        <v>56.391</v>
       </c>
       <c r="J57" s="1" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>0.56</t>
         </is>
       </c>
       <c r="K57" t="b">
@@ -3844,16 +3844,16 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>19</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Sydney Lamb</t>
+          <t>Ciara Lang</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>821897</v>
+        <v>906527</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -3889,34 +3889,34 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Raedyn Spademan</t>
+          <t>Sydney Lamb</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>816647</v>
+        <v>821897</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>5-5</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="G59" t="n">
-        <v>1743.8737</v>
+        <v>1723.5183</v>
       </c>
       <c r="H59" t="n">
         <v>1795.7245</v>
       </c>
       <c r="I59" t="n">
-        <v>51.851</v>
+        <v>72.206</v>
       </c>
       <c r="J59" s="1" t="inlineStr">
         <is>
-          <t>0.52</t>
+          <t>1.12</t>
         </is>
       </c>
       <c r="K59" t="b">
@@ -3934,16 +3934,16 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>18</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Shelby Laidlaw</t>
+          <t>Raedyn Spademan</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>816596</v>
+        <v>816647</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
@@ -3979,16 +3979,16 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>28</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Layla Matthew</t>
+          <t>Shelby Laidlaw</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>847129</v>
+        <v>816596</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
@@ -4024,16 +4024,16 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>15</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Keira Hurry</t>
+          <t>Layla Matthew</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>816275</v>
+        <v>847129</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
@@ -4041,17 +4041,17 @@
         </is>
       </c>
       <c r="G62" t="n">
+        <v>1743.8737</v>
+      </c>
+      <c r="H62" t="n">
         <v>1795.7245</v>
       </c>
-      <c r="H62" t="n">
-        <v>1877.0621</v>
-      </c>
       <c r="I62" t="n">
-        <v>81.33799999999999</v>
+        <v>51.851</v>
       </c>
       <c r="J62" s="1" t="inlineStr">
         <is>
-          <t>1.21</t>
+          <t>0.52</t>
         </is>
       </c>
       <c r="K62" t="b">
@@ -4069,16 +4069,16 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Kate Manness</t>
+          <t>Keira Hurry</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>835282</v>
+        <v>816275</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
@@ -4114,16 +4114,16 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>24</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Manon le Scodan</t>
+          <t>Kate Manness</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>811470</v>
+        <v>835282</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -4134,14 +4134,14 @@
         <v>1795.7245</v>
       </c>
       <c r="H64" t="n">
-        <v>1810.7957</v>
+        <v>1877.0621</v>
       </c>
       <c r="I64" t="n">
-        <v>15.071</v>
+        <v>81.33799999999999</v>
       </c>
       <c r="J64" s="1" t="inlineStr">
         <is>
-          <t>0.15</t>
+          <t>1.21</t>
         </is>
       </c>
       <c r="K64" t="b">
@@ -4159,16 +4159,16 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>21</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Sara Manness</t>
+          <t>Manon le Scodan</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>801530</v>
+        <v>811470</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
@@ -4204,16 +4204,16 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>26</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Kennedy Sisson</t>
+          <t>Sara Manness</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>891409</v>
+        <v>801530</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
@@ -4249,16 +4249,16 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>22</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Jessie Pellerin</t>
+          <t>Kennedy Sisson</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>801538</v>
+        <v>891409</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
@@ -4266,17 +4266,17 @@
         </is>
       </c>
       <c r="G67" t="n">
+        <v>1795.7245</v>
+      </c>
+      <c r="H67" t="n">
         <v>1810.7957</v>
       </c>
-      <c r="H67" t="n">
-        <v>1831.3744</v>
-      </c>
       <c r="I67" t="n">
-        <v>20.579</v>
+        <v>15.071</v>
       </c>
       <c r="J67" s="1" t="inlineStr">
         <is>
-          <t>0.21</t>
+          <t>0.15</t>
         </is>
       </c>
       <c r="K67" t="b">
@@ -4294,16 +4294,16 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>27</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Isa Goettl</t>
+          <t>Jessie Pellerin</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>816244</v>
+        <v>801538</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
@@ -4339,16 +4339,16 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Janelle Evans</t>
+          <t>Isa Goettl</t>
         </is>
       </c>
       <c r="E69" t="n">
-        <v>818654</v>
+        <v>816244</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
@@ -4384,16 +4384,16 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>17</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Kennedy Sisson</t>
+          <t>Janelle Evans</t>
         </is>
       </c>
       <c r="E70" t="n">
-        <v>891409</v>
+        <v>818654</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -4401,17 +4401,17 @@
         </is>
       </c>
       <c r="G70" t="n">
+        <v>1810.7957</v>
+      </c>
+      <c r="H70" t="n">
         <v>1831.3744</v>
       </c>
-      <c r="H70" t="n">
-        <v>1877.0621</v>
-      </c>
       <c r="I70" t="n">
-        <v>45.688</v>
+        <v>20.579</v>
       </c>
       <c r="J70" s="1" t="inlineStr">
         <is>
-          <t>0.46</t>
+          <t>0.21</t>
         </is>
       </c>
       <c r="K70" t="b">
@@ -4429,16 +4429,16 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>22</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Sara Manness</t>
+          <t>Kennedy Sisson</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>801530</v>
+        <v>891409</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
@@ -4474,16 +4474,16 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>26</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Manon le Scodan</t>
+          <t>Sara Manness</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>811470</v>
+        <v>801530</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
@@ -4519,16 +4519,16 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>21</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Morgan Walton</t>
+          <t>Manon le Scodan</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>822077</v>
+        <v>811470</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
@@ -4536,17 +4536,17 @@
         </is>
       </c>
       <c r="G73" t="n">
+        <v>1831.3744</v>
+      </c>
+      <c r="H73" t="n">
         <v>1877.0621</v>
       </c>
-      <c r="H73" t="n">
-        <v>1979.5911</v>
-      </c>
       <c r="I73" t="n">
-        <v>102.529</v>
+        <v>45.688</v>
       </c>
       <c r="J73" s="1" t="inlineStr">
         <is>
-          <t>1.43</t>
+          <t>0.46</t>
         </is>
       </c>
       <c r="K73" t="b">
@@ -4564,16 +4564,16 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Jaela Carter</t>
+          <t>Morgan Walton</t>
         </is>
       </c>
       <c r="E74" t="n">
-        <v>856721</v>
+        <v>822077</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -4609,16 +4609,16 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Layla Matthew</t>
+          <t>Jaela Carter</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>847129</v>
+        <v>856721</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
@@ -4654,16 +4654,16 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>15</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Raedyn Spademan</t>
+          <t>Layla Matthew</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>816647</v>
+        <v>847129</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
@@ -4699,16 +4699,16 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>18</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Shelby Laidlaw</t>
+          <t>Raedyn Spademan</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>816596</v>
+        <v>816647</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -4744,16 +4744,16 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>28</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Sydney Lamb</t>
+          <t>Shelby Laidlaw</t>
         </is>
       </c>
       <c r="E78" t="n">
-        <v>821897</v>
+        <v>816596</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
@@ -4761,17 +4761,17 @@
         </is>
       </c>
       <c r="G78" t="n">
+        <v>1877.0621</v>
+      </c>
+      <c r="H78" t="n">
         <v>1979.5911</v>
       </c>
-      <c r="H78" t="n">
-        <v>2039.6484</v>
-      </c>
       <c r="I78" t="n">
-        <v>60.057</v>
+        <v>102.529</v>
       </c>
       <c r="J78" s="1" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>1.43</t>
         </is>
       </c>
       <c r="K78" t="b">
@@ -4789,16 +4789,16 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Ciara Lang</t>
+          <t>Sydney Lamb</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>906527</v>
+        <v>821897</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -4834,16 +4834,16 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>19</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Isa Goettl</t>
+          <t>Ciara Lang</t>
         </is>
       </c>
       <c r="E80" t="n">
-        <v>816244</v>
+        <v>906527</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
@@ -4879,16 +4879,16 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Janelle Evans</t>
+          <t>Isa Goettl</t>
         </is>
       </c>
       <c r="E81" t="n">
-        <v>818654</v>
+        <v>816244</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
@@ -4924,16 +4924,16 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>17</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Jessie Pellerin</t>
+          <t>Janelle Evans</t>
         </is>
       </c>
       <c r="E82" t="n">
-        <v>801538</v>
+        <v>818654</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
@@ -4969,16 +4969,16 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>27</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Kate Manness</t>
+          <t>Jessie Pellerin</t>
         </is>
       </c>
       <c r="E83" t="n">
-        <v>835282</v>
+        <v>801538</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
@@ -4986,17 +4986,17 @@
         </is>
       </c>
       <c r="G83" t="n">
+        <v>1979.5911</v>
+      </c>
+      <c r="H83" t="n">
         <v>2039.6484</v>
       </c>
-      <c r="H83" t="n">
-        <v>2073.0542</v>
-      </c>
       <c r="I83" t="n">
-        <v>33.406</v>
+        <v>60.057</v>
       </c>
       <c r="J83" s="1" t="inlineStr">
         <is>
-          <t>0.33</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="K83" t="b">
@@ -5014,16 +5014,16 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>24</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Keira Hurry</t>
+          <t>Kate Manness</t>
         </is>
       </c>
       <c r="E84" t="n">
-        <v>816275</v>
+        <v>835282</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -5059,16 +5059,16 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Kennedy Sisson</t>
+          <t>Keira Hurry</t>
         </is>
       </c>
       <c r="E85" t="n">
-        <v>891409</v>
+        <v>816275</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
@@ -5104,16 +5104,16 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Manon le Scodan</t>
+          <t>Kennedy Sisson</t>
         </is>
       </c>
       <c r="E86" t="n">
-        <v>811470</v>
+        <v>891409</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>
@@ -5124,14 +5124,14 @@
         <v>2039.6484</v>
       </c>
       <c r="H86" t="n">
-        <v>2071.962</v>
+        <v>2073.0542</v>
       </c>
       <c r="I86" t="n">
-        <v>32.313</v>
+        <v>33.406</v>
       </c>
       <c r="J86" s="1" t="inlineStr">
         <is>
-          <t>0.32</t>
+          <t>0.33</t>
         </is>
       </c>
       <c r="K86" t="b">
@@ -5149,16 +5149,16 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>21</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Sara Manness</t>
+          <t>Manon le Scodan</t>
         </is>
       </c>
       <c r="E87" t="n">
-        <v>801530</v>
+        <v>811470</v>
       </c>
       <c r="F87" t="inlineStr">
         <is>
@@ -5169,14 +5169,14 @@
         <v>2039.6484</v>
       </c>
       <c r="H87" t="n">
-        <v>2073.0542</v>
+        <v>2071.962</v>
       </c>
       <c r="I87" t="n">
-        <v>33.406</v>
+        <v>32.313</v>
       </c>
       <c r="J87" s="1" t="inlineStr">
         <is>
-          <t>0.33</t>
+          <t>0.32</t>
         </is>
       </c>
       <c r="K87" t="b">
@@ -5194,16 +5194,16 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>26</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Gabrielle Lalonde</t>
+          <t>Sara Manness</t>
         </is>
       </c>
       <c r="E88" t="n">
-        <v>856725</v>
+        <v>801530</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
@@ -5211,17 +5211,17 @@
         </is>
       </c>
       <c r="G88" t="n">
-        <v>2071.962</v>
+        <v>2039.6484</v>
       </c>
       <c r="H88" t="n">
-        <v>2117.8325</v>
+        <v>2073.0542</v>
       </c>
       <c r="I88" t="n">
-        <v>45.871</v>
+        <v>33.406</v>
       </c>
       <c r="J88" s="1" t="inlineStr">
         <is>
-          <t>0.46</t>
+          <t>0.33</t>
         </is>
       </c>
       <c r="K88" t="b">
@@ -5239,16 +5239,16 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Kaitlyn Mallette</t>
+          <t>Gabrielle Lalonde</t>
         </is>
       </c>
       <c r="E89" t="n">
-        <v>847128</v>
+        <v>856725</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
@@ -5256,17 +5256,17 @@
         </is>
       </c>
       <c r="G89" t="n">
-        <v>2073.0542</v>
+        <v>2071.962</v>
       </c>
       <c r="H89" t="n">
-        <v>2130.694</v>
+        <v>2117.8325</v>
       </c>
       <c r="I89" t="n">
-        <v>57.64</v>
+        <v>45.871</v>
       </c>
       <c r="J89" s="1" t="inlineStr">
         <is>
-          <t>0.58</t>
+          <t>0.46</t>
         </is>
       </c>
       <c r="K89" t="b">
@@ -5284,16 +5284,16 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>11</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Morgan Walton</t>
+          <t>Kaitlyn Mallette</t>
         </is>
       </c>
       <c r="E90" t="n">
-        <v>822077</v>
+        <v>847128</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
@@ -5329,16 +5329,16 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Abby Richardson</t>
+          <t>Morgan Walton</t>
         </is>
       </c>
       <c r="E91" t="n">
-        <v>824230</v>
+        <v>822077</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -5349,14 +5349,14 @@
         <v>2073.0542</v>
       </c>
       <c r="H91" t="n">
-        <v>2130.2207</v>
+        <v>2130.694</v>
       </c>
       <c r="I91" t="n">
-        <v>57.167</v>
+        <v>57.64</v>
       </c>
       <c r="J91" s="1" t="inlineStr">
         <is>
-          <t>0.57</t>
+          <t>0.58</t>
         </is>
       </c>
       <c r="K91" t="b">
@@ -5374,16 +5374,16 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Paige Wallace</t>
+          <t>Abby Richardson</t>
         </is>
       </c>
       <c r="E92" t="n">
-        <v>822075</v>
+        <v>824230</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -5419,16 +5419,16 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Layla Matthew</t>
+          <t>Paige Wallace</t>
         </is>
       </c>
       <c r="E93" t="n">
-        <v>847129</v>
+        <v>822075</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
@@ -5436,17 +5436,17 @@
         </is>
       </c>
       <c r="G93" t="n">
-        <v>2117.8325</v>
+        <v>2073.0542</v>
       </c>
       <c r="H93" t="n">
-        <v>2172.0796</v>
+        <v>2130.2207</v>
       </c>
       <c r="I93" t="n">
-        <v>54.247</v>
+        <v>57.167</v>
       </c>
       <c r="J93" s="1" t="inlineStr">
         <is>
-          <t>0.54</t>
+          <t>0.57</t>
         </is>
       </c>
       <c r="K93" t="b">
@@ -5464,16 +5464,16 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>15</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Raedyn Spademan</t>
+          <t>Layla Matthew</t>
         </is>
       </c>
       <c r="E94" t="n">
-        <v>816647</v>
+        <v>847129</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
@@ -5481,13 +5481,13 @@
         </is>
       </c>
       <c r="G94" t="n">
-        <v>2130.2207</v>
+        <v>2117.8325</v>
       </c>
       <c r="H94" t="n">
-        <v>2184.5713</v>
+        <v>2172.0796</v>
       </c>
       <c r="I94" t="n">
-        <v>54.351</v>
+        <v>54.247</v>
       </c>
       <c r="J94" s="1" t="inlineStr">
         <is>
@@ -5509,16 +5509,16 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>18</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Shelby Laidlaw</t>
+          <t>Raedyn Spademan</t>
         </is>
       </c>
       <c r="E95" t="n">
-        <v>816596</v>
+        <v>816647</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
@@ -5529,14 +5529,14 @@
         <v>2130.2207</v>
       </c>
       <c r="H95" t="n">
-        <v>2177.6528</v>
+        <v>2184.5713</v>
       </c>
       <c r="I95" t="n">
-        <v>47.432</v>
+        <v>54.351</v>
       </c>
       <c r="J95" s="1" t="inlineStr">
         <is>
-          <t>0.47</t>
+          <t>0.54</t>
         </is>
       </c>
       <c r="K95" t="b">
@@ -5554,16 +5554,16 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>28</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Sydney Lamb</t>
+          <t>Shelby Laidlaw</t>
         </is>
       </c>
       <c r="E96" t="n">
-        <v>821897</v>
+        <v>816596</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
@@ -5571,17 +5571,17 @@
         </is>
       </c>
       <c r="G96" t="n">
-        <v>2130.694</v>
+        <v>2130.2207</v>
       </c>
       <c r="H96" t="n">
-        <v>2166.533</v>
+        <v>2177.6528</v>
       </c>
       <c r="I96" t="n">
-        <v>35.839</v>
+        <v>47.432</v>
       </c>
       <c r="J96" s="1" t="inlineStr">
         <is>
-          <t>0.36</t>
+          <t>0.47</t>
         </is>
       </c>
       <c r="K96" t="b">
@@ -5599,16 +5599,16 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Ciara Lang</t>
+          <t>Sydney Lamb</t>
         </is>
       </c>
       <c r="E97" t="n">
-        <v>906527</v>
+        <v>821897</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
@@ -5644,16 +5644,16 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>19</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Keira Hurry</t>
+          <t>Ciara Lang</t>
         </is>
       </c>
       <c r="E98" t="n">
-        <v>816275</v>
+        <v>906527</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
@@ -5661,17 +5661,17 @@
         </is>
       </c>
       <c r="G98" t="n">
+        <v>2130.694</v>
+      </c>
+      <c r="H98" t="n">
         <v>2166.533</v>
       </c>
-      <c r="H98" t="n">
-        <v>2235.609</v>
-      </c>
       <c r="I98" t="n">
-        <v>69.07599999999999</v>
+        <v>35.839</v>
       </c>
       <c r="J98" s="1" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>0.36</t>
         </is>
       </c>
       <c r="K98" t="b">
@@ -5689,16 +5689,16 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Kate Manness</t>
+          <t>Keira Hurry</t>
         </is>
       </c>
       <c r="E99" t="n">
-        <v>835282</v>
+        <v>816275</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -5734,16 +5734,16 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>24</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Isa Goettl</t>
+          <t>Kate Manness</t>
         </is>
       </c>
       <c r="E100" t="n">
-        <v>816244</v>
+        <v>835282</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
@@ -5751,17 +5751,17 @@
         </is>
       </c>
       <c r="G100" t="n">
-        <v>2172.0796</v>
+        <v>2166.533</v>
       </c>
       <c r="H100" t="n">
-        <v>2242.3623</v>
+        <v>2235.609</v>
       </c>
       <c r="I100" t="n">
-        <v>70.283</v>
+        <v>69.07599999999999</v>
       </c>
       <c r="J100" s="1" t="inlineStr">
         <is>
-          <t>1.10</t>
+          <t>1.09</t>
         </is>
       </c>
       <c r="K100" t="b">
@@ -5779,16 +5779,16 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Jessie Pellerin</t>
+          <t>Isa Goettl</t>
         </is>
       </c>
       <c r="E101" t="n">
-        <v>801538</v>
+        <v>816244</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -5796,17 +5796,17 @@
         </is>
       </c>
       <c r="G101" t="n">
-        <v>2177.6528</v>
+        <v>2172.0796</v>
       </c>
       <c r="H101" t="n">
-        <v>2235.738</v>
+        <v>2242.3623</v>
       </c>
       <c r="I101" t="n">
-        <v>58.085</v>
+        <v>70.283</v>
       </c>
       <c r="J101" s="1" t="inlineStr">
         <is>
-          <t>0.58</t>
+          <t>1.10</t>
         </is>
       </c>
       <c r="K101" t="b">
@@ -5824,16 +5824,16 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>27</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Janelle Evans</t>
+          <t>Jessie Pellerin</t>
         </is>
       </c>
       <c r="E102" t="n">
-        <v>818654</v>
+        <v>801538</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
@@ -5841,17 +5841,17 @@
         </is>
       </c>
       <c r="G102" t="n">
-        <v>2184.5713</v>
+        <v>2177.6528</v>
       </c>
       <c r="H102" t="n">
-        <v>2233.9497</v>
+        <v>2235.738</v>
       </c>
       <c r="I102" t="n">
-        <v>49.378</v>
+        <v>58.085</v>
       </c>
       <c r="J102" s="1" t="inlineStr">
         <is>
-          <t>0.49</t>
+          <t>0.58</t>
         </is>
       </c>
       <c r="K102" t="b">
@@ -5869,16 +5869,16 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>17</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Sara Manness</t>
+          <t>Janelle Evans</t>
         </is>
       </c>
       <c r="E103" t="n">
-        <v>801530</v>
+        <v>818654</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
@@ -5886,17 +5886,17 @@
         </is>
       </c>
       <c r="G103" t="n">
+        <v>2184.5713</v>
+      </c>
+      <c r="H103" t="n">
         <v>2233.9497</v>
       </c>
-      <c r="H103" t="n">
-        <v>2302.9822</v>
-      </c>
       <c r="I103" t="n">
-        <v>69.032</v>
+        <v>49.378</v>
       </c>
       <c r="J103" s="1" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>0.49</t>
         </is>
       </c>
       <c r="K103" t="b">
@@ -5914,16 +5914,16 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>26</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Jaela Carter</t>
+          <t>Sara Manness</t>
         </is>
       </c>
       <c r="E104" t="n">
-        <v>856721</v>
+        <v>801530</v>
       </c>
       <c r="F104" t="inlineStr">
         <is>
@@ -5931,17 +5931,17 @@
         </is>
       </c>
       <c r="G104" t="n">
-        <v>2235.609</v>
+        <v>2233.9497</v>
       </c>
       <c r="H104" t="n">
-        <v>2323.7222</v>
+        <v>2302.9822</v>
       </c>
       <c r="I104" t="n">
-        <v>88.113</v>
+        <v>69.032</v>
       </c>
       <c r="J104" s="1" t="inlineStr">
         <is>
-          <t>1.28</t>
+          <t>1.09</t>
         </is>
       </c>
       <c r="K104" t="b">
@@ -5959,16 +5959,16 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Morgan Walton</t>
+          <t>Jaela Carter</t>
         </is>
       </c>
       <c r="E105" t="n">
-        <v>822077</v>
+        <v>856721</v>
       </c>
       <c r="F105" t="inlineStr">
         <is>
@@ -5979,14 +5979,14 @@
         <v>2235.609</v>
       </c>
       <c r="H105" t="n">
-        <v>2290.4434</v>
+        <v>2323.7222</v>
       </c>
       <c r="I105" t="n">
-        <v>54.834</v>
+        <v>88.113</v>
       </c>
       <c r="J105" s="1" t="inlineStr">
         <is>
-          <t>0.55</t>
+          <t>1.28</t>
         </is>
       </c>
       <c r="K105" t="b">
@@ -6004,16 +6004,16 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Kennedy Sisson</t>
+          <t>Morgan Walton</t>
         </is>
       </c>
       <c r="E106" t="n">
-        <v>891409</v>
+        <v>822077</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
@@ -6021,17 +6021,17 @@
         </is>
       </c>
       <c r="G106" t="n">
-        <v>2235.738</v>
+        <v>2235.609</v>
       </c>
       <c r="H106" t="n">
-        <v>2320.1516</v>
+        <v>2290.4434</v>
       </c>
       <c r="I106" t="n">
-        <v>84.414</v>
+        <v>54.834</v>
       </c>
       <c r="J106" s="1" t="inlineStr">
         <is>
-          <t>1.24</t>
+          <t>0.55</t>
         </is>
       </c>
       <c r="K106" t="b">
@@ -6049,16 +6049,16 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Manon le Scodan</t>
+          <t>Kennedy Sisson</t>
         </is>
       </c>
       <c r="E107" t="n">
-        <v>811470</v>
+        <v>891409</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
@@ -6066,17 +6066,17 @@
         </is>
       </c>
       <c r="G107" t="n">
-        <v>2242.3623</v>
+        <v>2235.738</v>
       </c>
       <c r="H107" t="n">
-        <v>2298.7224</v>
+        <v>2320.1516</v>
       </c>
       <c r="I107" t="n">
-        <v>56.36</v>
+        <v>84.414</v>
       </c>
       <c r="J107" s="1" t="inlineStr">
         <is>
-          <t>0.56</t>
+          <t>1.24</t>
         </is>
       </c>
       <c r="K107" t="b">
@@ -6094,16 +6094,16 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>21</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Ciara Lang</t>
+          <t>Manon le Scodan</t>
         </is>
       </c>
       <c r="E108" t="n">
-        <v>906527</v>
+        <v>811470</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -6111,17 +6111,17 @@
         </is>
       </c>
       <c r="G108" t="n">
-        <v>2290.4434</v>
+        <v>2242.3623</v>
       </c>
       <c r="H108" t="n">
-        <v>2339.7053</v>
+        <v>2298.7224</v>
       </c>
       <c r="I108" t="n">
-        <v>49.262</v>
+        <v>56.36</v>
       </c>
       <c r="J108" s="1" t="inlineStr">
         <is>
-          <t>0.49</t>
+          <t>0.56</t>
         </is>
       </c>
       <c r="K108" t="b">
@@ -6139,36 +6139,38 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>19</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Senkova Aneta</t>
+          <t>Ciara Lang</t>
         </is>
       </c>
       <c r="E109" t="n">
-        <v>801351</v>
+        <v>906527</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>5-5</t>
         </is>
       </c>
       <c r="G109" t="n">
-        <v>1200.5223</v>
-      </c>
-      <c r="H109" t="inlineStr"/>
+        <v>2290.4434</v>
+      </c>
+      <c r="H109" t="n">
+        <v>2339.7053</v>
+      </c>
       <c r="I109" t="n">
-        <v>1199.478</v>
+        <v>49.262</v>
       </c>
       <c r="J109" s="1" t="inlineStr">
         <is>
-          <t>19.59</t>
+          <t>0.49</t>
         </is>
       </c>
       <c r="K109" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110">
@@ -6201,7 +6203,9 @@
       <c r="G110" t="n">
         <v>2298.7224</v>
       </c>
-      <c r="H110" t="inlineStr"/>
+      <c r="H110" t="n">
+        <v>2400</v>
+      </c>
       <c r="I110" t="n">
         <v>101.278</v>
       </c>
@@ -6211,7 +6215,7 @@
         </is>
       </c>
       <c r="K110" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="111">
@@ -6244,7 +6248,9 @@
       <c r="G111" t="n">
         <v>2302.9822</v>
       </c>
-      <c r="H111" t="inlineStr"/>
+      <c r="H111" t="n">
+        <v>2400</v>
+      </c>
       <c r="I111" t="n">
         <v>97.018</v>
       </c>
@@ -6254,7 +6260,7 @@
         </is>
       </c>
       <c r="K111" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="112">
@@ -6287,7 +6293,9 @@
       <c r="G112" t="n">
         <v>2320.1516</v>
       </c>
-      <c r="H112" t="inlineStr"/>
+      <c r="H112" t="n">
+        <v>2400</v>
+      </c>
       <c r="I112" t="n">
         <v>79.848</v>
       </c>
@@ -6297,7 +6305,7 @@
         </is>
       </c>
       <c r="K112" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113">
@@ -6330,7 +6338,9 @@
       <c r="G113" t="n">
         <v>2323.7222</v>
       </c>
-      <c r="H113" t="inlineStr"/>
+      <c r="H113" t="n">
+        <v>2400</v>
+      </c>
       <c r="I113" t="n">
         <v>76.27800000000001</v>
       </c>
@@ -6340,7 +6350,7 @@
         </is>
       </c>
       <c r="K113" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="114">
@@ -6373,7 +6383,9 @@
       <c r="G114" t="n">
         <v>2339.7053</v>
       </c>
-      <c r="H114" t="inlineStr"/>
+      <c r="H114" t="n">
+        <v>2400</v>
+      </c>
       <c r="I114" t="n">
         <v>60.295</v>
       </c>
@@ -6383,7 +6395,7 @@
         </is>
       </c>
       <c r="K114" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -6562,7 +6574,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-10-02T23:24:07.512207+00:00</t>
+          <t>2026-10-02T23:24:59.008691+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>